<commit_message>
update GW 38 2025/26
</commit_message>
<xml_diff>
--- a/app/team_stats_2025.xlsx
+++ b/app/team_stats_2025.xlsx
@@ -558,10 +558,10 @@
         <v>30</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J2" s="1" t="n">
         <v>5</v>
@@ -570,13 +570,13 @@
         <v>3</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M2" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N2" s="1" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O2" s="1" t="n">
         <v>7</v>
@@ -585,7 +585,7 @@
         <v>5</v>
       </c>
       <c r="Q2" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -615,7 +615,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>7</v>
@@ -624,13 +624,13 @@
         <v>5</v>
       </c>
       <c r="K3" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>14</v>
@@ -639,10 +639,10 @@
         <v>10</v>
       </c>
       <c r="P3" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q3" s="1" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -657,13 +657,13 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>10</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>3</v>
@@ -687,13 +687,13 @@
         <v>-4</v>
       </c>
       <c r="M4" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N4" s="1" t="n">
         <v>17</v>
       </c>
       <c r="O4" s="1" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P4" s="1" t="n">
         <v>12</v>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>14</v>
@@ -723,10 +723,10 @@
         <v>3</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H5" s="1" t="n">
         <v>19</v>
@@ -744,7 +744,7 @@
         <v>11</v>
       </c>
       <c r="M5" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N5" s="1" t="n">
         <v>23</v>
@@ -753,10 +753,10 @@
         <v>9</v>
       </c>
       <c r="P5" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q5" s="1" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -786,10 +786,10 @@
         <v>15</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J6" s="1" t="n">
         <v>8</v>
@@ -798,13 +798,13 @@
         <v>4</v>
       </c>
       <c r="L6" s="1" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M6" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N6" s="1" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O6" s="1" t="n">
         <v>11</v>
@@ -813,7 +813,7 @@
         <v>7</v>
       </c>
       <c r="Q6" s="1" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -885,7 +885,7 @@
         <v>22</v>
       </c>
       <c r="H9" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I9" s="1" t="n">
         <v>6</v>
@@ -894,13 +894,13 @@
         <v>5</v>
       </c>
       <c r="K9" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="M9" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N9" s="1" t="n">
         <v>21</v>
@@ -909,10 +909,10 @@
         <v>6</v>
       </c>
       <c r="P9" s="1" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q9" s="1" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -942,7 +942,7 @@
         <v>47</v>
       </c>
       <c r="H10" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I10" s="1" t="n">
         <v>12</v>
@@ -951,13 +951,13 @@
         <v>1</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="1" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M10" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N10" s="1" t="n">
         <v>31</v>
@@ -966,10 +966,10 @@
         <v>1</v>
       </c>
       <c r="P10" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="1" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11">
@@ -984,10 +984,10 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>1</v>
@@ -996,7 +996,7 @@
         <v>2</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H11" s="1" t="n">
         <v>19</v>
@@ -1014,10 +1014,10 @@
         <v>13</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N11" s="1" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O11" s="1" t="n">
         <v>5</v>
@@ -1026,7 +1026,7 @@
         <v>6</v>
       </c>
       <c r="Q11" s="1" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="C23" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D23" s="1" t="n">
         <v>9</v>
@@ -1533,10 +1533,10 @@
         <v>5</v>
       </c>
       <c r="F23" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="1" t="n">
         <v>4</v>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>5</v>
       </c>
       <c r="H23" s="1" t="n">
         <v>19</v>
@@ -1554,7 +1554,7 @@
         <v>14</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>20</v>
@@ -1563,10 +1563,10 @@
         <v>10</v>
       </c>
       <c r="P23" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q23" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24">
@@ -1596,13 +1596,13 @@
         <v>34</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I24" s="1" t="n">
         <v>13</v>
       </c>
       <c r="J24" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K24" s="1" t="n">
         <v>3</v>
@@ -1611,13 +1611,13 @@
         <v>20</v>
       </c>
       <c r="M24" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N24" s="1" t="n">
         <v>27</v>
       </c>
       <c r="O24" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P24" s="1" t="n">
         <v>5</v>
@@ -1653,13 +1653,13 @@
         <v>19</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I25" s="1" t="n">
         <v>9</v>
       </c>
       <c r="J25" s="1" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K25" s="1" t="n">
         <v>5</v>
@@ -1668,13 +1668,13 @@
         <v>8</v>
       </c>
       <c r="M25" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N25" s="1" t="n">
         <v>19</v>
       </c>
       <c r="O25" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P25" s="1" t="n">
         <v>7</v>
@@ -1695,10 +1695,10 @@
         </is>
       </c>
       <c r="C26" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E26" s="1" t="n">
         <v>6</v>
@@ -1707,7 +1707,7 @@
         <v>5</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26" s="1" t="n">
         <v>19</v>
@@ -1725,10 +1725,10 @@
         <v>-1</v>
       </c>
       <c r="M26" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N26" s="1" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O26" s="1" t="n">
         <v>12</v>
@@ -1737,7 +1737,7 @@
         <v>12</v>
       </c>
       <c r="Q26" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1752,10 +1752,10 @@
         </is>
       </c>
       <c r="C27" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>4</v>
@@ -1764,7 +1764,7 @@
         <v>2</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H27" s="1" t="n">
         <v>19</v>
@@ -1782,10 +1782,10 @@
         <v>7</v>
       </c>
       <c r="M27" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N27" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O27" s="1" t="n">
         <v>7</v>
@@ -1794,7 +1794,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="1" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28">
@@ -1824,10 +1824,10 @@
         <v>23</v>
       </c>
       <c r="H28" s="1" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J28" s="1" t="n">
         <v>1</v>
@@ -1836,13 +1836,13 @@
         <v>8</v>
       </c>
       <c r="L28" s="1" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M28" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N28" s="1" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O28" s="1" t="n">
         <v>4</v>
@@ -1851,7 +1851,7 @@
         <v>11</v>
       </c>
       <c r="Q28" s="1" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29">

</xml_diff>